<commit_message>
v1.2.2 Llenado de la primera columna
</commit_message>
<xml_diff>
--- a/output/PRADIVO WORLD COMPANY 1096.xlsx
+++ b/output/PRADIVO WORLD COMPANY 1096.xlsx
@@ -5,44 +5,26 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maric\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maric\Desktop\auto\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D5344E1-86A8-4B80-B6DC-B1CE9449EB5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89CB4C9A-EEC6-4FFB-B705-73019C23D216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{6F36AFD9-B07A-4120-8C17-9B9B96AC2EF3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IMPO118" sheetId="1" r:id="rId1"/>
     <sheet name="IMPO235" sheetId="2" r:id="rId2"/>
     <sheet name="EXPO118" sheetId="3" r:id="rId3"/>
     <sheet name="EXPO235" sheetId="4" r:id="rId4"/>
+    <sheet name="PRADIVO WORLD COMPANY 1096" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="54">
   <si>
     <t>N°</t>
   </si>
@@ -83,10 +65,127 @@
     <t>ESTADO (MULTA)</t>
   </si>
   <si>
+    <t>01-118-1-2026- 1606</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 1867</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 1848</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 2022</t>
+  </si>
+  <si>
     <t>FECHA Y HORA DE  TRANSMISION AGTE. DE CARGA</t>
   </si>
   <si>
     <t>FECHA Y HORA DE TERMINO DE EMBARQUE</t>
+  </si>
+  <si>
+    <t>Manifiesto de Carga</t>
+  </si>
+  <si>
+    <t>Fecha del Manifiesto de Carga</t>
+  </si>
+  <si>
+    <t>Manifiesto Desconsolidado</t>
+  </si>
+  <si>
+    <t>Fecha del Manifiesto Desconsolidado</t>
+  </si>
+  <si>
+    <t>Agente de Carga RUC</t>
+  </si>
+  <si>
+    <t>Número de Ticket</t>
+  </si>
+  <si>
+    <t>Fecha de Llegada</t>
+  </si>
+  <si>
+    <t>Fecha de Término de la Descarga</t>
+  </si>
+  <si>
+    <t>Estado del Manifiesto Desconsolidado</t>
+  </si>
+  <si>
+    <t>15/06/2026 12:16:52</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 32157</t>
+  </si>
+  <si>
+    <t>07/07/2026 17:16:28</t>
+  </si>
+  <si>
+    <t>20602733808</t>
+  </si>
+  <si>
+    <t>2026-44033906</t>
+  </si>
+  <si>
+    <t>17/07/2026 07:36:00</t>
+  </si>
+  <si>
+    <t>18/07/2026 16:00:00</t>
+  </si>
+  <si>
+    <t>NUMERADO</t>
+  </si>
+  <si>
+    <t>10/07/2026 14:12:18</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 33970</t>
+  </si>
+  <si>
+    <t>16/07/2026 15:08:54</t>
+  </si>
+  <si>
+    <t>2026-46115963</t>
+  </si>
+  <si>
+    <t>26/07/2026 19:15:00</t>
+  </si>
+  <si>
+    <t>27/07/2026 21:19:00</t>
+  </si>
+  <si>
+    <t>08/07/2026 14:32:49</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 35652</t>
+  </si>
+  <si>
+    <t>30/07/2026 19:05:48</t>
+  </si>
+  <si>
+    <t>2026-49651564</t>
+  </si>
+  <si>
+    <t>05/08/2026 22:40:00</t>
+  </si>
+  <si>
+    <t>06/08/2026 14:18:00</t>
+  </si>
+  <si>
+    <t>25/07/2026 19:32:43</t>
+  </si>
+  <si>
+    <t>01-118-1-2026- 35925</t>
+  </si>
+  <si>
+    <t>30/07/2026 19:34:32</t>
+  </si>
+  <si>
+    <t>2026-49655561</t>
+  </si>
+  <si>
+    <t>06/08/2026 16:24:00</t>
+  </si>
+  <si>
+    <t>...</t>
   </si>
 </sst>
 </file>
@@ -504,11 +603,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05289A66-F660-4D3D-BBFC-B812FC1D9810}">
-  <dimension ref="A1:M1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,6 +649,26 @@
       </c>
       <c r="M1" s="1" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -555,11 +677,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84F711BF-FB44-48D0-AC5C-C466CD98967A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -603,11 +725,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69585CB0-9F9B-40BB-BE0C-31222A672CCB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -627,10 +749,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>12</v>
@@ -642,11 +764,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB726D33-E6FC-42A3-B62A-EDE71ADD2F2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -666,10 +788,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>12</v>
@@ -678,4 +800,162 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v1.2.5 3 columnas listo
</commit_message>
<xml_diff>
--- a/output/PRADIVO WORLD COMPANY 1096.xlsx
+++ b/output/PRADIVO WORLD COMPANY 1096.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maric\Desktop\auto\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E87AAA10-81B6-4E32-BB34-CECA010816B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A40909A-C35D-4614-9389-DB5D009D87E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IMPO118" sheetId="1" r:id="rId1"/>
@@ -68,15 +68,27 @@
     <t>01-118-1-2026- 1606</t>
   </si>
   <si>
+    <t>17/07/2026 07:36:00</t>
+  </si>
+  <si>
     <t>01-118-1-2026- 1867</t>
   </si>
   <si>
+    <t>26/07/2026 19:15:00</t>
+  </si>
+  <si>
     <t>01-118-1-2026- 1848</t>
   </si>
   <si>
+    <t>05/08/2026 22:40:00</t>
+  </si>
+  <si>
     <t>01-118-1-2026- 2022</t>
   </si>
   <si>
+    <t>06/08/2026 16:24:00</t>
+  </si>
+  <si>
     <t>FECHA Y HORA DE  TRANSMISION AGTE. DE CARGA</t>
   </si>
   <si>
@@ -125,9 +137,6 @@
     <t>2026-44033906</t>
   </si>
   <si>
-    <t>17/07/2026 07:36:00</t>
-  </si>
-  <si>
     <t>18/07/2026 16:00:00</t>
   </si>
   <si>
@@ -146,9 +155,6 @@
     <t>2026-46115963</t>
   </si>
   <si>
-    <t>26/07/2026 19:15:00</t>
-  </si>
-  <si>
     <t>27/07/2026 21:19:00</t>
   </si>
   <si>
@@ -164,9 +170,6 @@
     <t>2026-49651564</t>
   </si>
   <si>
-    <t>05/08/2026 22:40:00</t>
-  </si>
-  <si>
     <t>06/08/2026 14:18:00</t>
   </si>
   <si>
@@ -180,9 +183,6 @@
   </si>
   <si>
     <t>2026-49655561</t>
-  </si>
-  <si>
-    <t>06/08/2026 16:24:00</t>
   </si>
   <si>
     <t>...</t>
@@ -609,6 +609,7 @@
   <cols>
     <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -730,10 +731,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>12</v>
@@ -769,10 +770,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>12</v>
@@ -801,31 +802,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -833,115 +834,115 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" t="s">
         <v>38</v>
-      </c>
-      <c r="E3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" t="s">
-        <v>39</v>
-      </c>
-      <c r="G3" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G4" t="s">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="H4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="H5" t="s">
         <v>53</v>
       </c>
       <c r="I5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>